<commit_message>
fix(ci): resolve ruff RUF019 and stale workbook integrity cache (#8)
* fix(ci): resolve ruff RUF019 in typed constitution cascade

* fix(ecosystem): correct future-dated log entry and refresh cached workbook status

The first Daily Writing Log row carried a 2027-01-01 placeholder date while holding session word counts, so the Config future-entry check (B28) flagged it once CI read the cached values. Set the date to 2026-10-11 to match the following session rows and refresh the cached integrity cells (B28, B33, C33). Fix the same placeholder date in the ecosystem template workbook.

---------

Co-authored-by: 3u2t <3u2t@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Master_Writing_Ecosystem.xlsx
+++ b/Master_Writing_Ecosystem.xlsx
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B28" s="14">
         <f ca="1">COUNTIFS('Daily Writing Log'!$A$5:$A$34,"&gt;"&amp;$A$2,'Daily Writing Log'!$H$5:$H$34,"&gt;0")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>96</v>
@@ -12267,11 +12267,11 @@
       </c>
       <c r="B33" s="45">
         <f ca="1">COUNTIF(B25:B32,"&lt;&gt;0")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C33" s="44" t="str">
         <f ca="1">IF(B33=0,"✅ All 8 integrity checks pass","⚠️ "&amp;B33&amp;" check(s) need attention")</f>
-        <v>⚠️ 1 check(s) need attention</v>
+        <v>✅ All 8 integrity checks pass</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="11.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -17617,7 +17617,7 @@
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88">
-        <v>46388</v>
+        <v>46306</v>
       </c>
       <c r="B5" s="89" t="s">
         <v>122</v>

</xml_diff>